<commit_message>
Supplementary Table 1: add colony details and approximate coordinates
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/supplement/Supplementary Table 1.xlsx
+++ b/supplement/Supplementary Table 1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I13"/>
+  <dimension ref="A1:K15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -425,6 +425,8 @@
     <col width="18" customWidth="1" min="7" max="7"/>
     <col width="52" customWidth="1" min="8" max="8"/>
     <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -473,6 +475,16 @@
           <t>Origin</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Latitude (approx.)</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Longitude (approx.)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -511,6 +523,12 @@
           <t>Obuasi, Ghana</t>
         </is>
       </c>
+      <c r="J2" t="n">
+        <v>6.21</v>
+      </c>
+      <c r="K2" t="n">
+        <v>-1.69</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -552,6 +570,12 @@
           <t>Siaya county, western Kenya</t>
         </is>
       </c>
+      <c r="J3" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="K3" t="n">
+        <v>34.2</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -590,6 +614,12 @@
           <t>Siaya county, western Kenya</t>
         </is>
       </c>
+      <c r="J4" t="n">
+        <v>-0.06</v>
+      </c>
+      <c r="K4" t="n">
+        <v>34.2</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -628,6 +658,12 @@
           <t>Kisumu, western Kenya</t>
         </is>
       </c>
+      <c r="J5" t="n">
+        <v>-0.1</v>
+      </c>
+      <c r="K5" t="n">
+        <v>34.75</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -669,6 +705,12 @@
           <t>Vallee du Kou 7, Houet, Burkina Faso</t>
         </is>
       </c>
+      <c r="J6" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="K6" t="n">
+        <v>-4.39</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -707,6 +749,12 @@
           <t>Vallee du Kou 7, Houet, Burkina Faso</t>
         </is>
       </c>
+      <c r="J7" t="n">
+        <v>11.39</v>
+      </c>
+      <c r="K7" t="n">
+        <v>-4.39</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -745,6 +793,12 @@
           <t>Banfora district, Comoe, Burkina Faso</t>
         </is>
       </c>
+      <c r="J8" t="n">
+        <v>10.62</v>
+      </c>
+      <c r="K8" t="n">
+        <v>-4.56</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -783,6 +837,12 @@
           <t>Tiassale, Cote d'Ivoire</t>
         </is>
       </c>
+      <c r="J9" t="n">
+        <v>5.9</v>
+      </c>
+      <c r="K9" t="n">
+        <v>-4.82</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -821,6 +881,12 @@
           <t>Yaounde, Cameroon</t>
         </is>
       </c>
+      <c r="J10" t="n">
+        <v>3.87</v>
+      </c>
+      <c r="K10" t="n">
+        <v>11.52</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -859,6 +925,12 @@
           <t>Gaoua district, Poni, Burkina Faso</t>
         </is>
       </c>
+      <c r="J11" t="n">
+        <v>10.33</v>
+      </c>
+      <c r="K11" t="n">
+        <v>-3.18</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -897,6 +969,12 @@
           <t>Chokwe, southern Mozambique</t>
         </is>
       </c>
+      <c r="J12" t="n">
+        <v>-24.49</v>
+      </c>
+      <c r="K12" t="n">
+        <v>32.86</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -933,6 +1011,19 @@
       <c r="I13" t="inlineStr">
         <is>
           <t>Upper River Region, The Gambia</t>
+        </is>
+      </c>
+      <c r="J13" t="n">
+        <v>13.31</v>
+      </c>
+      <c r="K13" t="n">
+        <v>-14.21</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Coordinates are approximate (decimal degrees): the centre of the named locality, taken from OpenStreetMap place records, not the exact collection site. Tiassale agrees with the MalariaGEN field record (5.898, -4.823). Siaya is the county centre. The Gambia is Basse Santa Su, Upper River Region.</t>
         </is>
       </c>
     </row>

</xml_diff>